<commit_message>
Configuracion de MCPs de postgres y powerBI
</commit_message>
<xml_diff>
--- a/pentaho/mis_procesos/data/xlsx/Proyecto_BI - Metas Seguros AltaVista.xlsx
+++ b/pentaho/mis_procesos/data/xlsx/Proyecto_BI - Metas Seguros AltaVista.xlsx
@@ -3,7 +3,8 @@
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
   <workbookPr/>
   <sheets>
-    <sheet state="visible" name="Vale viendolo mejor, creo que p" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Ver con Segmentos de cliente" sheetId="1" r:id="rId5"/>
+    <sheet state="visible" name="Ver sin Segmentos" sheetId="2" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr/>
@@ -11,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="71">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="206" uniqueCount="71">
   <si>
     <t>anio</t>
   </si>
@@ -326,8 +327,14 @@
       </border>
     </dxf>
   </dxfs>
-  <tableStyles count="1">
-    <tableStyle count="4" pivot="0" name="Vale viendolo mejor, creo que p-style">
+  <tableStyles count="2">
+    <tableStyle count="4" pivot="0" name="Ver con Segmentos de cliente-style">
+      <tableStyleElement dxfId="1" type="headerRow"/>
+      <tableStyleElement dxfId="2" type="firstRowStripe"/>
+      <tableStyleElement dxfId="3" type="secondRowStripe"/>
+      <tableStyleElement dxfId="4" size="0" type="wholeTable"/>
+    </tableStyle>
+    <tableStyle count="4" pivot="0" name="Ver sin Segmentos-style">
       <tableStyleElement dxfId="1" type="headerRow"/>
       <tableStyleElement dxfId="2" type="firstRowStripe"/>
       <tableStyleElement dxfId="3" type="secondRowStripe"/>
@@ -338,6 +345,10 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:cx="http://schemas.microsoft.com/office/drawing/2014/chartex" xmlns:cx1="http://schemas.microsoft.com/office/drawing/2015/9/8/chartex" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:dgm="http://schemas.openxmlformats.org/drawingml/2006/diagram" xmlns:x3Unk="http://schemas.microsoft.com/office/drawing/2010/slicer" xmlns:sle15="http://schemas.microsoft.com/office/drawing/2012/slicer"/>
 </file>
 
@@ -356,7 +367,22 @@
     <tableColumn name="meta_renovacion" id="6"/>
     <tableColumn name="meta_asegurados" id="7"/>
   </tableColumns>
-  <tableStyleInfo name="Vale viendolo mejor, creo que p-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+  <tableStyleInfo name="Ver con Segmentos de cliente-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
+</table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" ref="A1:G33" displayName="Metas_Seguros_Alta_Vista_2" name="Metas_Seguros_Alta_Vista_2" id="2">
+  <tableColumns count="7">
+    <tableColumn name="anio" id="1"/>
+    <tableColumn name="cod_producto" id="2"/>
+    <tableColumn name="segmento_cliente" id="3"/>
+    <tableColumn name="nro_contrato_referencia" id="4"/>
+    <tableColumn name="monto_meta_ingreso" id="5"/>
+    <tableColumn name="meta_renovacion" id="6"/>
+    <tableColumn name="meta_asegurados" id="7"/>
+  </tableColumns>
+  <tableStyleInfo name="Ver sin Segmentos-style" showColumnStripes="0" showFirstColumn="1" showLastColumn="1" showRowStripes="1"/>
 </table>
 </file>
 
@@ -2070,4 +2096,786 @@
     <tablePart r:id="rId3"/>
   </tableParts>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mx="http://schemas.microsoft.com/office/mac/excel/2008/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:mv="urn:schemas-microsoft-com:mac:vml" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="0" summaryRight="0"/>
+  </sheetPr>
+  <sheetFormatPr customHeight="1" defaultColWidth="12.63" defaultRowHeight="15.75"/>
+  <cols>
+    <col customWidth="1" min="2" max="2" width="18.75"/>
+    <col customWidth="1" min="3" max="3" width="21.75"/>
+    <col customWidth="1" min="4" max="4" width="27.38"/>
+    <col customWidth="1" min="5" max="5" width="22.38"/>
+    <col customWidth="1" min="6" max="6" width="19.5"/>
+    <col customWidth="1" min="7" max="7" width="21.13"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="22.5" customHeight="1">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" ht="22.5" customHeight="1">
+      <c r="A2" s="2">
+        <v>2018.0</v>
+      </c>
+      <c r="B2" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2" s="2">
+        <v>145.0</v>
+      </c>
+      <c r="E2" s="2" t="s">
+        <v>8</v>
+      </c>
+      <c r="F2" s="2">
+        <v>120.0</v>
+      </c>
+      <c r="G2" s="2">
+        <v>85.0</v>
+      </c>
+    </row>
+    <row r="3" ht="22.5" customHeight="1">
+      <c r="A3" s="2">
+        <v>2018.0</v>
+      </c>
+      <c r="B3" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C3" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D3" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="E3" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="F3" s="2">
+        <v>280.0</v>
+      </c>
+      <c r="G3" s="2">
+        <v>140.0</v>
+      </c>
+    </row>
+    <row r="4" ht="22.5" customHeight="1">
+      <c r="A4" s="2">
+        <v>2018.0</v>
+      </c>
+      <c r="B4" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C4" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D4" s="2">
+        <v>1340.0</v>
+      </c>
+      <c r="E4" s="2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F4" s="2">
+        <v>190.0</v>
+      </c>
+      <c r="G4" s="2">
+        <v>100.0</v>
+      </c>
+    </row>
+    <row r="5" ht="22.5" customHeight="1">
+      <c r="A5" s="2">
+        <v>2018.0</v>
+      </c>
+      <c r="B5" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C5" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D5" s="2">
+        <v>442.0</v>
+      </c>
+      <c r="E5" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="F5" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="G5" s="2">
+        <v>25.0</v>
+      </c>
+    </row>
+    <row r="6" ht="22.5" customHeight="1">
+      <c r="A6" s="2">
+        <v>2019.0</v>
+      </c>
+      <c r="B6" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C6" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D6" s="2">
+        <v>911.0</v>
+      </c>
+      <c r="E6" s="2" t="s">
+        <v>18</v>
+      </c>
+      <c r="F6" s="2">
+        <v>155.0</v>
+      </c>
+      <c r="G6" s="2">
+        <v>95.0</v>
+      </c>
+    </row>
+    <row r="7" ht="22.5" customHeight="1">
+      <c r="A7" s="2">
+        <v>2019.0</v>
+      </c>
+      <c r="B7" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C7" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D7" s="2">
+        <v>92.0</v>
+      </c>
+      <c r="E7" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="F7" s="2">
+        <v>290.0</v>
+      </c>
+      <c r="G7" s="2">
+        <v>150.0</v>
+      </c>
+    </row>
+    <row r="8" ht="22.5" customHeight="1">
+      <c r="A8" s="2">
+        <v>2019.0</v>
+      </c>
+      <c r="B8" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C8" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D8" s="2">
+        <v>1405.0</v>
+      </c>
+      <c r="E8" s="2" t="s">
+        <v>21</v>
+      </c>
+      <c r="F8" s="2">
+        <v>200.0</v>
+      </c>
+      <c r="G8" s="2">
+        <v>110.0</v>
+      </c>
+    </row>
+    <row r="9" ht="22.5" customHeight="1">
+      <c r="A9" s="2">
+        <v>2019.0</v>
+      </c>
+      <c r="B9" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C9" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D9" s="2">
+        <v>1980.0</v>
+      </c>
+      <c r="E9" s="2" t="s">
+        <v>23</v>
+      </c>
+      <c r="F9" s="2">
+        <v>50.0</v>
+      </c>
+      <c r="G9" s="2">
+        <v>25.0</v>
+      </c>
+    </row>
+    <row r="10" ht="22.5" customHeight="1">
+      <c r="A10" s="2">
+        <v>2020.0</v>
+      </c>
+      <c r="B10" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C10" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D10" s="2">
+        <v>250.0</v>
+      </c>
+      <c r="E10" s="2" t="s">
+        <v>25</v>
+      </c>
+      <c r="F10" s="2">
+        <v>135.0</v>
+      </c>
+      <c r="G10" s="2">
+        <v>92.0</v>
+      </c>
+    </row>
+    <row r="11" ht="22.5" customHeight="1">
+      <c r="A11" s="2">
+        <v>2020.0</v>
+      </c>
+      <c r="B11" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C11" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D11" s="2">
+        <v>1150.0</v>
+      </c>
+      <c r="E11" s="2" t="s">
+        <v>27</v>
+      </c>
+      <c r="F11" s="2">
+        <v>320.0</v>
+      </c>
+      <c r="G11" s="2">
+        <v>170.0</v>
+      </c>
+    </row>
+    <row r="12" ht="22.5" customHeight="1">
+      <c r="A12" s="2">
+        <v>2020.0</v>
+      </c>
+      <c r="B12" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C12" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D12" s="2">
+        <v>230.0</v>
+      </c>
+      <c r="E12" s="2" t="s">
+        <v>30</v>
+      </c>
+      <c r="F12" s="2">
+        <v>235.0</v>
+      </c>
+      <c r="G12" s="2">
+        <v>125.0</v>
+      </c>
+    </row>
+    <row r="13" ht="22.5" customHeight="1">
+      <c r="A13" s="2">
+        <v>2020.0</v>
+      </c>
+      <c r="B13" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C13" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D13" s="2">
+        <v>490.0</v>
+      </c>
+      <c r="E13" s="2" t="s">
+        <v>32</v>
+      </c>
+      <c r="F13" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="G13" s="2">
+        <v>32.0</v>
+      </c>
+    </row>
+    <row r="14" ht="22.5" customHeight="1">
+      <c r="A14" s="2">
+        <v>2020.0</v>
+      </c>
+      <c r="B14" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="C14" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D14" s="2">
+        <v>12.0</v>
+      </c>
+      <c r="E14" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="F14" s="2">
+        <v>430.0</v>
+      </c>
+      <c r="G14" s="2">
+        <v>300.0</v>
+      </c>
+    </row>
+    <row r="15" ht="22.5" customHeight="1">
+      <c r="A15" s="2">
+        <v>2020.0</v>
+      </c>
+      <c r="B15" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="C15" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D15" s="2">
+        <v>812.0</v>
+      </c>
+      <c r="E15" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="F15" s="2">
+        <v>190.0</v>
+      </c>
+      <c r="G15" s="2">
+        <v>105.0</v>
+      </c>
+    </row>
+    <row r="16" ht="22.5" customHeight="1">
+      <c r="A16" s="2">
+        <v>2021.0</v>
+      </c>
+      <c r="B16" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C16" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D16" s="2">
+        <v>980.0</v>
+      </c>
+      <c r="E16" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="F16" s="2">
+        <v>165.0</v>
+      </c>
+      <c r="G16" s="2">
+        <v>102.0</v>
+      </c>
+    </row>
+    <row r="17" ht="22.5" customHeight="1">
+      <c r="A17" s="2">
+        <v>2021.0</v>
+      </c>
+      <c r="B17" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C17" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D17" s="2">
+        <v>321.0</v>
+      </c>
+      <c r="E17" s="2" t="s">
+        <v>40</v>
+      </c>
+      <c r="F17" s="2">
+        <v>330.0</v>
+      </c>
+      <c r="G17" s="2">
+        <v>180.0</v>
+      </c>
+    </row>
+    <row r="18" ht="22.5" customHeight="1">
+      <c r="A18" s="2">
+        <v>2021.0</v>
+      </c>
+      <c r="B18" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C18" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D18" s="2">
+        <v>280.0</v>
+      </c>
+      <c r="E18" s="2" t="s">
+        <v>42</v>
+      </c>
+      <c r="F18" s="2">
+        <v>245.0</v>
+      </c>
+      <c r="G18" s="2">
+        <v>135.0</v>
+      </c>
+    </row>
+    <row r="19" ht="22.5" customHeight="1">
+      <c r="A19" s="2">
+        <v>2021.0</v>
+      </c>
+      <c r="B19" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C19" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D19" s="2">
+        <v>2000.0</v>
+      </c>
+      <c r="E19" s="2" t="s">
+        <v>43</v>
+      </c>
+      <c r="F19" s="2">
+        <v>60.0</v>
+      </c>
+      <c r="G19" s="2">
+        <v>30.0</v>
+      </c>
+    </row>
+    <row r="20" ht="22.5" customHeight="1">
+      <c r="A20" s="2">
+        <v>2021.0</v>
+      </c>
+      <c r="B20" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="C20" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D20" s="2">
+        <v>99.0</v>
+      </c>
+      <c r="E20" s="2" t="s">
+        <v>46</v>
+      </c>
+      <c r="F20" s="2">
+        <v>475.0</v>
+      </c>
+      <c r="G20" s="2">
+        <v>340.0</v>
+      </c>
+    </row>
+    <row r="21" ht="22.5" customHeight="1">
+      <c r="A21" s="2">
+        <v>2021.0</v>
+      </c>
+      <c r="B21" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="C21" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D21" s="2">
+        <v>850.0</v>
+      </c>
+      <c r="E21" s="2" t="s">
+        <v>48</v>
+      </c>
+      <c r="F21" s="2">
+        <v>205.0</v>
+      </c>
+      <c r="G21" s="2">
+        <v>115.0</v>
+      </c>
+    </row>
+    <row r="22" ht="22.5" customHeight="1">
+      <c r="A22" s="2">
+        <v>2022.0</v>
+      </c>
+      <c r="B22" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C22" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D22" s="2">
+        <v>1601.0</v>
+      </c>
+      <c r="E22" s="2" t="s">
+        <v>49</v>
+      </c>
+      <c r="F22" s="2">
+        <v>160.0</v>
+      </c>
+      <c r="G22" s="2">
+        <v>100.0</v>
+      </c>
+    </row>
+    <row r="23" ht="22.5" customHeight="1">
+      <c r="A23" s="2">
+        <v>2022.0</v>
+      </c>
+      <c r="B23" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C23" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D23" s="2">
+        <v>1280.0</v>
+      </c>
+      <c r="E23" s="2" t="s">
+        <v>51</v>
+      </c>
+      <c r="F23" s="2">
+        <v>360.0</v>
+      </c>
+      <c r="G23" s="2">
+        <v>195.0</v>
+      </c>
+    </row>
+    <row r="24" ht="22.5" customHeight="1">
+      <c r="A24" s="2">
+        <v>2022.0</v>
+      </c>
+      <c r="B24" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C24" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D24" s="2">
+        <v>1111.0</v>
+      </c>
+      <c r="E24" s="2" t="s">
+        <v>53</v>
+      </c>
+      <c r="F24" s="2">
+        <v>250.0</v>
+      </c>
+      <c r="G24" s="2">
+        <v>140.0</v>
+      </c>
+    </row>
+    <row r="25" ht="22.5" customHeight="1">
+      <c r="A25" s="2">
+        <v>2022.0</v>
+      </c>
+      <c r="B25" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D25" s="2">
+        <v>1900.0</v>
+      </c>
+      <c r="E25" s="2" t="s">
+        <v>55</v>
+      </c>
+      <c r="F25" s="2">
+        <v>65.0</v>
+      </c>
+      <c r="G25" s="2">
+        <v>33.0</v>
+      </c>
+    </row>
+    <row r="26" ht="22.5" customHeight="1">
+      <c r="A26" s="2">
+        <v>2022.0</v>
+      </c>
+      <c r="B26" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D26" s="2">
+        <v>140.0</v>
+      </c>
+      <c r="E26" s="2" t="s">
+        <v>58</v>
+      </c>
+      <c r="F26" s="2">
+        <v>495.0</v>
+      </c>
+      <c r="G26" s="2">
+        <v>365.0</v>
+      </c>
+    </row>
+    <row r="27" ht="22.5" customHeight="1">
+      <c r="A27" s="2">
+        <v>2022.0</v>
+      </c>
+      <c r="B27" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D27" s="2">
+        <v>890.0</v>
+      </c>
+      <c r="E27" s="2" t="s">
+        <v>60</v>
+      </c>
+      <c r="F27" s="2">
+        <v>220.0</v>
+      </c>
+      <c r="G27" s="2">
+        <v>125.0</v>
+      </c>
+    </row>
+    <row r="28" ht="22.5" customHeight="1">
+      <c r="A28" s="2">
+        <v>2023.0</v>
+      </c>
+      <c r="B28" s="2">
+        <v>1.0</v>
+      </c>
+      <c r="C28" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D28" s="2">
+        <v>1650.0</v>
+      </c>
+      <c r="E28" s="2" t="s">
+        <v>61</v>
+      </c>
+      <c r="F28" s="2">
+        <v>170.0</v>
+      </c>
+      <c r="G28" s="2">
+        <v>110.0</v>
+      </c>
+    </row>
+    <row r="29" ht="22.5" customHeight="1">
+      <c r="A29" s="2">
+        <v>2023.0</v>
+      </c>
+      <c r="B29" s="2">
+        <v>2.0</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D29" s="2">
+        <v>2000.0</v>
+      </c>
+      <c r="E29" s="2" t="s">
+        <v>63</v>
+      </c>
+      <c r="F29" s="2">
+        <v>380.0</v>
+      </c>
+      <c r="G29" s="2">
+        <v>210.0</v>
+      </c>
+    </row>
+    <row r="30" ht="22.5" customHeight="1">
+      <c r="A30" s="2">
+        <v>2023.0</v>
+      </c>
+      <c r="B30" s="2">
+        <v>3.0</v>
+      </c>
+      <c r="C30" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D30" s="2">
+        <v>350.0</v>
+      </c>
+      <c r="E30" s="2" t="s">
+        <v>65</v>
+      </c>
+      <c r="F30" s="2">
+        <v>285.0</v>
+      </c>
+      <c r="G30" s="2">
+        <v>165.0</v>
+      </c>
+    </row>
+    <row r="31" ht="22.5" customHeight="1">
+      <c r="A31" s="2">
+        <v>2023.0</v>
+      </c>
+      <c r="B31" s="2">
+        <v>4.0</v>
+      </c>
+      <c r="C31" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D31" s="2">
+        <v>1950.0</v>
+      </c>
+      <c r="E31" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="F31" s="2">
+        <v>75.0</v>
+      </c>
+      <c r="G31" s="2">
+        <v>42.0</v>
+      </c>
+    </row>
+    <row r="32" ht="22.5" customHeight="1">
+      <c r="A32" s="2">
+        <v>2023.0</v>
+      </c>
+      <c r="B32" s="2">
+        <v>5.0</v>
+      </c>
+      <c r="C32" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D32" s="2">
+        <v>190.0</v>
+      </c>
+      <c r="E32" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="F32" s="2">
+        <v>520.0</v>
+      </c>
+      <c r="G32" s="2">
+        <v>390.0</v>
+      </c>
+    </row>
+    <row r="33" ht="22.5" customHeight="1">
+      <c r="A33" s="2">
+        <v>2023.0</v>
+      </c>
+      <c r="B33" s="2">
+        <v>6.0</v>
+      </c>
+      <c r="C33" s="2" t="s">
+        <v>9</v>
+      </c>
+      <c r="D33" s="2">
+        <v>1675.0</v>
+      </c>
+      <c r="E33" s="2" t="s">
+        <v>70</v>
+      </c>
+      <c r="F33" s="2">
+        <v>200.0</v>
+      </c>
+      <c r="G33" s="2">
+        <v>120.0</v>
+      </c>
+    </row>
+  </sheetData>
+  <drawing r:id="rId1"/>
+  <tableParts count="1">
+    <tablePart r:id="rId3"/>
+  </tableParts>
+</worksheet>
 </file>
</xml_diff>